<commit_message>
add test for decorator report_to_file
</commit_message>
<xml_diff>
--- a/data/operations_for_test.xlsx
+++ b/data/operations_for_test.xlsx
@@ -459,10 +459,7 @@
       <c r="O2" s="4" t="n">
         <v>160.89</v>
       </c>
-      <c r="P2" s="1" t="n">
-        <f aca="false">SUM(O2:O3)</f>
-        <v>224.89</v>
-      </c>
+      <c r="P2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">

</xml_diff>